<commit_message>
Update portfolio-updates.xlsx on 2025-12-14 13:01:36
</commit_message>
<xml_diff>
--- a/portfolio-updates.xlsx
+++ b/portfolio-updates.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D120"/>
+  <dimension ref="A1:D121"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2249,6 +2249,22 @@
         <v>298.0499877929688</v>
       </c>
     </row>
+    <row r="121">
+      <c r="A121" t="inlineStr">
+        <is>
+          <t>2025-12-14</t>
+        </is>
+      </c>
+      <c r="B121" t="n">
+        <v>53.02000045776367</v>
+      </c>
+      <c r="C121" t="n">
+        <v>347.4500122070312</v>
+      </c>
+      <c r="D121" t="n">
+        <v>298.0499877929688</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update portfolio-updates.xlsx on 2025-12-15 13:11:47
</commit_message>
<xml_diff>
--- a/portfolio-updates.xlsx
+++ b/portfolio-updates.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D121"/>
+  <dimension ref="A1:D122"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2265,6 +2265,19 @@
         <v>298.0499877929688</v>
       </c>
     </row>
+    <row r="122">
+      <c r="A122" t="inlineStr">
+        <is>
+          <t>2025-12-15</t>
+        </is>
+      </c>
+      <c r="B122" t="n">
+        <v>53.13999938964844</v>
+      </c>
+      <c r="C122" t="n">
+        <v>298.4500122070312</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update portfolio-updates.xlsx on 2025-12-16 13:10:00
</commit_message>
<xml_diff>
--- a/portfolio-updates.xlsx
+++ b/portfolio-updates.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D122"/>
+  <dimension ref="A1:D123"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2278,6 +2278,19 @@
         <v>298.4500122070312</v>
       </c>
     </row>
+    <row r="123">
+      <c r="A123" t="inlineStr">
+        <is>
+          <t>2025-12-16</t>
+        </is>
+      </c>
+      <c r="B123" t="n">
+        <v>52.66999816894531</v>
+      </c>
+      <c r="C123" t="n">
+        <v>284.4500122070312</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update portfolio-updates.xlsx on 2025-12-17 13:09:45
</commit_message>
<xml_diff>
--- a/portfolio-updates.xlsx
+++ b/portfolio-updates.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D123"/>
+  <dimension ref="A1:D124"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2291,6 +2291,19 @@
         <v>284.4500122070312</v>
       </c>
     </row>
+    <row r="124">
+      <c r="A124" t="inlineStr">
+        <is>
+          <t>2025-12-17</t>
+        </is>
+      </c>
+      <c r="B124" t="n">
+        <v>51.93999862670898</v>
+      </c>
+      <c r="C124" t="n">
+        <v>284.4500122070312</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update portfolio-updates.xlsx on 2025-12-18 13:08:28
</commit_message>
<xml_diff>
--- a/portfolio-updates.xlsx
+++ b/portfolio-updates.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D124"/>
+  <dimension ref="A1:D125"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2304,6 +2304,19 @@
         <v>284.4500122070312</v>
       </c>
     </row>
+    <row r="125">
+      <c r="A125" t="inlineStr">
+        <is>
+          <t>2025-12-18</t>
+        </is>
+      </c>
+      <c r="B125" t="n">
+        <v>51.77999877929688</v>
+      </c>
+      <c r="C125" t="n">
+        <v>284.75</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update portfolio-updates.xlsx on 2025-12-19 13:06:40
</commit_message>
<xml_diff>
--- a/portfolio-updates.xlsx
+++ b/portfolio-updates.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D125"/>
+  <dimension ref="A1:D126"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2317,6 +2317,19 @@
         <v>284.75</v>
       </c>
     </row>
+    <row r="126">
+      <c r="A126" t="inlineStr">
+        <is>
+          <t>2025-12-19</t>
+        </is>
+      </c>
+      <c r="B126" t="n">
+        <v>52.59000015258789</v>
+      </c>
+      <c r="C126" t="n">
+        <v>286.0499877929688</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update portfolio-updates.xlsx on 2025-12-20 13:01:28
</commit_message>
<xml_diff>
--- a/portfolio-updates.xlsx
+++ b/portfolio-updates.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D126"/>
+  <dimension ref="A1:D127"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2330,6 +2330,22 @@
         <v>286.0499877929688</v>
       </c>
     </row>
+    <row r="127">
+      <c r="A127" t="inlineStr">
+        <is>
+          <t>2025-12-20</t>
+        </is>
+      </c>
+      <c r="B127" t="n">
+        <v>52.59000015258789</v>
+      </c>
+      <c r="C127" t="n">
+        <v>352.6499938964844</v>
+      </c>
+      <c r="D127" t="n">
+        <v>286.0499877929688</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update portfolio-updates.xlsx on 2025-12-21 13:01:56
</commit_message>
<xml_diff>
--- a/portfolio-updates.xlsx
+++ b/portfolio-updates.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D127"/>
+  <dimension ref="A1:D128"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2346,6 +2346,22 @@
         <v>286.0499877929688</v>
       </c>
     </row>
+    <row r="128">
+      <c r="A128" t="inlineStr">
+        <is>
+          <t>2025-12-21</t>
+        </is>
+      </c>
+      <c r="B128" t="n">
+        <v>52.59000015258789</v>
+      </c>
+      <c r="C128" t="n">
+        <v>352.6499938964844</v>
+      </c>
+      <c r="D128" t="n">
+        <v>286.0499877929688</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update portfolio-updates.xlsx on 2025-12-22 13:06:53
</commit_message>
<xml_diff>
--- a/portfolio-updates.xlsx
+++ b/portfolio-updates.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D128"/>
+  <dimension ref="A1:D129"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2362,6 +2362,19 @@
         <v>286.0499877929688</v>
       </c>
     </row>
+    <row r="129">
+      <c r="A129" t="inlineStr">
+        <is>
+          <t>2025-12-22</t>
+        </is>
+      </c>
+      <c r="B129" t="n">
+        <v>53.5099983215332</v>
+      </c>
+      <c r="C129" t="n">
+        <v>286.7000122070312</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update portfolio-updates.xlsx on 2025-12-23 13:08:35
</commit_message>
<xml_diff>
--- a/portfolio-updates.xlsx
+++ b/portfolio-updates.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D129"/>
+  <dimension ref="A1:D130"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2375,6 +2375,19 @@
         <v>286.7000122070312</v>
       </c>
     </row>
+    <row r="130">
+      <c r="A130" t="inlineStr">
+        <is>
+          <t>2025-12-23</t>
+        </is>
+      </c>
+      <c r="B130" t="n">
+        <v>53.61999893188477</v>
+      </c>
+      <c r="C130" t="n">
+        <v>284.3500061035156</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update portfolio-updates.xlsx on 2025-12-24 13:06:03
</commit_message>
<xml_diff>
--- a/portfolio-updates.xlsx
+++ b/portfolio-updates.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D130"/>
+  <dimension ref="A1:D131"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2388,6 +2388,19 @@
         <v>284.3500061035156</v>
       </c>
     </row>
+    <row r="131">
+      <c r="A131" t="inlineStr">
+        <is>
+          <t>2025-12-24</t>
+        </is>
+      </c>
+      <c r="B131" t="n">
+        <v>53.29999923706055</v>
+      </c>
+      <c r="C131" t="n">
+        <v>284.8500061035156</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update portfolio-updates.xlsx on 2025-12-25 13:05:52
</commit_message>
<xml_diff>
--- a/portfolio-updates.xlsx
+++ b/portfolio-updates.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D131"/>
+  <dimension ref="A1:D132"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2401,6 +2401,19 @@
         <v>284.8500061035156</v>
       </c>
     </row>
+    <row r="132">
+      <c r="A132" t="inlineStr">
+        <is>
+          <t>2025-12-25</t>
+        </is>
+      </c>
+      <c r="B132" t="n">
+        <v>53.29999923706055</v>
+      </c>
+      <c r="C132" t="n">
+        <v>284.6000061035156</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update portfolio-updates.xlsx on 2025-12-26 13:05:58
</commit_message>
<xml_diff>
--- a/portfolio-updates.xlsx
+++ b/portfolio-updates.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D132"/>
+  <dimension ref="A1:D133"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2414,6 +2414,19 @@
         <v>284.6000061035156</v>
       </c>
     </row>
+    <row r="133">
+      <c r="A133" t="inlineStr">
+        <is>
+          <t>2025-12-26</t>
+        </is>
+      </c>
+      <c r="B133" t="n">
+        <v>53.20000076293945</v>
+      </c>
+      <c r="C133" t="n">
+        <v>281.75</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update portfolio-updates.xlsx on 2025-12-27 13:03:13
</commit_message>
<xml_diff>
--- a/portfolio-updates.xlsx
+++ b/portfolio-updates.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D133"/>
+  <dimension ref="A1:D134"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2427,6 +2427,19 @@
         <v>281.75</v>
       </c>
     </row>
+    <row r="134">
+      <c r="A134" t="inlineStr">
+        <is>
+          <t>2025-12-27</t>
+        </is>
+      </c>
+      <c r="B134" t="n">
+        <v>53.20000076293945</v>
+      </c>
+      <c r="C134" t="n">
+        <v>281.75</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update portfolio-updates.xlsx on 2025-12-28 13:04:04
</commit_message>
<xml_diff>
--- a/portfolio-updates.xlsx
+++ b/portfolio-updates.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D134"/>
+  <dimension ref="A1:D135"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2440,6 +2440,19 @@
         <v>281.75</v>
       </c>
     </row>
+    <row r="135">
+      <c r="A135" t="inlineStr">
+        <is>
+          <t>2025-12-28</t>
+        </is>
+      </c>
+      <c r="B135" t="n">
+        <v>53.20000076293945</v>
+      </c>
+      <c r="C135" t="n">
+        <v>281.75</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update portfolio-updates.xlsx on 2025-12-29 13:09:50
</commit_message>
<xml_diff>
--- a/portfolio-updates.xlsx
+++ b/portfolio-updates.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D135"/>
+  <dimension ref="A1:D136"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2453,6 +2453,19 @@
         <v>281.75</v>
       </c>
     </row>
+    <row r="136">
+      <c r="A136" t="inlineStr">
+        <is>
+          <t>2025-12-29</t>
+        </is>
+      </c>
+      <c r="B136" t="n">
+        <v>52.72999954223633</v>
+      </c>
+      <c r="C136" t="n">
+        <v>282.8500061035156</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update portfolio-updates.xlsx on 2025-12-30 13:08:39
</commit_message>
<xml_diff>
--- a/portfolio-updates.xlsx
+++ b/portfolio-updates.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D136"/>
+  <dimension ref="A1:D137"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2466,6 +2466,19 @@
         <v>282.8500061035156</v>
       </c>
     </row>
+    <row r="137">
+      <c r="A137" t="inlineStr">
+        <is>
+          <t>2025-12-30</t>
+        </is>
+      </c>
+      <c r="B137" t="n">
+        <v>52</v>
+      </c>
+      <c r="C137" t="n">
+        <v>277.1000061035156</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update portfolio-updates.xlsx on 2025-12-31 13:06:46
</commit_message>
<xml_diff>
--- a/portfolio-updates.xlsx
+++ b/portfolio-updates.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D137"/>
+  <dimension ref="A1:D138"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2479,6 +2479,19 @@
         <v>277.1000061035156</v>
       </c>
     </row>
+    <row r="138">
+      <c r="A138" t="inlineStr">
+        <is>
+          <t>2025-12-31</t>
+        </is>
+      </c>
+      <c r="B138" t="n">
+        <v>52.66999816894531</v>
+      </c>
+      <c r="C138" t="n">
+        <v>278.0499877929688</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update portfolio-updates.xlsx on 2026-01-01 13:07:05
</commit_message>
<xml_diff>
--- a/portfolio-updates.xlsx
+++ b/portfolio-updates.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D138"/>
+  <dimension ref="A1:D139"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2492,6 +2492,19 @@
         <v>278.0499877929688</v>
       </c>
     </row>
+    <row r="139">
+      <c r="A139" t="inlineStr">
+        <is>
+          <t>2026-01-01</t>
+        </is>
+      </c>
+      <c r="B139" t="n">
+        <v>52.47000122070312</v>
+      </c>
+      <c r="C139" t="n">
+        <v>283.7999877929688</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>